<commit_message>
suppression modaliteentree et sortie 8dadb362ba7224847d7dde3edb817d24d16b89ae
</commit_message>
<xml_diff>
--- a/422-contenu-fhir---mise-à-jour-du-séjour/ig/StructureDefinition-tddui-encounter-sejour.xlsx
+++ b/422-contenu-fhir---mise-à-jour-du-séjour/ig/StructureDefinition-tddui-encounter-sejour.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4038" uniqueCount="644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4038" uniqueCount="642">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-11T15:25:25+00:00</t>
+    <t>2026-02-16T10:05:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1752,9 +1752,6 @@
     <t>http://hl7.org/fhir/ValueSet/encounter-admit-source|4.0.1</t>
   </si>
   <si>
-    <t>provenance</t>
-  </si>
-  <si>
     <t>.admissionReferralSourceCode</t>
   </si>
   <si>
@@ -1880,9 +1877,6 @@
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/encounter-discharge-disposition|4.0.1</t>
-  </si>
-  <si>
-    <t>motifSortie</t>
   </si>
   <si>
     <t>.dischargeDispositionCode</t>
@@ -13188,27 +13182,27 @@
         <v>102</v>
       </c>
       <c r="AK93" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL93" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM93" t="s" s="2">
         <v>554</v>
       </c>
-      <c r="AL93" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM93" t="s" s="2">
+      <c r="AN93" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO93" t="s" s="2">
         <v>555</v>
-      </c>
-      <c r="AN93" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO93" t="s" s="2">
-        <v>556</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -13234,10 +13228,10 @@
         <v>225</v>
       </c>
       <c r="L94" t="s" s="2">
+        <v>557</v>
+      </c>
+      <c r="M94" t="s" s="2">
         <v>558</v>
-      </c>
-      <c r="M94" t="s" s="2">
-        <v>559</v>
       </c>
       <c r="N94" s="2"/>
       <c r="O94" s="2"/>
@@ -13267,11 +13261,11 @@
         <v>336</v>
       </c>
       <c r="Y94" t="s" s="2">
+        <v>559</v>
+      </c>
+      <c r="Z94" t="s" s="2">
         <v>560</v>
       </c>
-      <c r="Z94" t="s" s="2">
-        <v>561</v>
-      </c>
       <c r="AA94" t="s" s="2">
         <v>81</v>
       </c>
@@ -13288,7 +13282,7 @@
         <v>81</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>79</v>
@@ -13315,15 +13309,15 @@
         <v>81</v>
       </c>
       <c r="AO94" t="s" s="2">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -13349,16 +13343,16 @@
         <v>225</v>
       </c>
       <c r="L95" t="s" s="2">
+        <v>563</v>
+      </c>
+      <c r="M95" t="s" s="2">
         <v>564</v>
       </c>
-      <c r="M95" t="s" s="2">
+      <c r="N95" t="s" s="2">
         <v>565</v>
       </c>
-      <c r="N95" t="s" s="2">
+      <c r="O95" t="s" s="2">
         <v>566</v>
-      </c>
-      <c r="O95" t="s" s="2">
-        <v>567</v>
       </c>
       <c r="P95" t="s" s="2">
         <v>81</v>
@@ -13386,11 +13380,11 @@
         <v>336</v>
       </c>
       <c r="Y95" t="s" s="2">
+        <v>567</v>
+      </c>
+      <c r="Z95" t="s" s="2">
         <v>568</v>
       </c>
-      <c r="Z95" t="s" s="2">
-        <v>569</v>
-      </c>
       <c r="AA95" t="s" s="2">
         <v>81</v>
       </c>
@@ -13407,7 +13401,7 @@
         <v>81</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>79</v>
@@ -13428,21 +13422,21 @@
         <v>81</v>
       </c>
       <c r="AM95" t="s" s="2">
+        <v>569</v>
+      </c>
+      <c r="AN95" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO95" t="s" s="2">
         <v>570</v>
-      </c>
-      <c r="AN95" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO95" t="s" s="2">
-        <v>571</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -13468,10 +13462,10 @@
         <v>225</v>
       </c>
       <c r="L96" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>573</v>
-      </c>
-      <c r="M96" t="s" s="2">
-        <v>574</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" s="2"/>
@@ -13501,11 +13495,11 @@
         <v>114</v>
       </c>
       <c r="Y96" t="s" s="2">
+        <v>574</v>
+      </c>
+      <c r="Z96" t="s" s="2">
         <v>575</v>
       </c>
-      <c r="Z96" t="s" s="2">
-        <v>576</v>
-      </c>
       <c r="AA96" t="s" s="2">
         <v>81</v>
       </c>
@@ -13522,7 +13516,7 @@
         <v>81</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>79</v>
@@ -13543,21 +13537,21 @@
         <v>81</v>
       </c>
       <c r="AM96" t="s" s="2">
+        <v>576</v>
+      </c>
+      <c r="AN96" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO96" t="s" s="2">
         <v>577</v>
-      </c>
-      <c r="AN96" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO96" t="s" s="2">
-        <v>578</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13583,10 +13577,10 @@
         <v>225</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>579</v>
+      </c>
+      <c r="M97" t="s" s="2">
         <v>580</v>
-      </c>
-      <c r="M97" t="s" s="2">
-        <v>581</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" s="2"/>
@@ -13616,11 +13610,11 @@
         <v>114</v>
       </c>
       <c r="Y97" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="Z97" t="s" s="2">
         <v>582</v>
       </c>
-      <c r="Z97" t="s" s="2">
-        <v>583</v>
-      </c>
       <c r="AA97" t="s" s="2">
         <v>81</v>
       </c>
@@ -13637,7 +13631,7 @@
         <v>81</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>79</v>
@@ -13658,21 +13652,21 @@
         <v>81</v>
       </c>
       <c r="AM97" t="s" s="2">
+        <v>583</v>
+      </c>
+      <c r="AN97" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO97" t="s" s="2">
         <v>584</v>
-      </c>
-      <c r="AN97" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO97" t="s" s="2">
-        <v>585</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -13695,13 +13689,13 @@
         <v>81</v>
       </c>
       <c r="K98" t="s" s="2">
+        <v>586</v>
+      </c>
+      <c r="L98" t="s" s="2">
         <v>587</v>
       </c>
-      <c r="L98" t="s" s="2">
+      <c r="M98" t="s" s="2">
         <v>588</v>
-      </c>
-      <c r="M98" t="s" s="2">
-        <v>589</v>
       </c>
       <c r="N98" s="2"/>
       <c r="O98" s="2"/>
@@ -13752,7 +13746,7 @@
         <v>81</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>79</v>
@@ -13773,21 +13767,21 @@
         <v>81</v>
       </c>
       <c r="AM98" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="AN98" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO98" t="s" s="2">
         <v>590</v>
-      </c>
-      <c r="AN98" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO98" t="s" s="2">
-        <v>591</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13813,10 +13807,10 @@
         <v>225</v>
       </c>
       <c r="L99" t="s" s="2">
+        <v>592</v>
+      </c>
+      <c r="M99" t="s" s="2">
         <v>593</v>
-      </c>
-      <c r="M99" t="s" s="2">
-        <v>594</v>
       </c>
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
@@ -13846,11 +13840,11 @@
         <v>336</v>
       </c>
       <c r="Y99" t="s" s="2">
+        <v>594</v>
+      </c>
+      <c r="Z99" t="s" s="2">
         <v>595</v>
       </c>
-      <c r="Z99" t="s" s="2">
-        <v>596</v>
-      </c>
       <c r="AA99" t="s" s="2">
         <v>81</v>
       </c>
@@ -13867,7 +13861,7 @@
         <v>81</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>79</v>
@@ -13882,27 +13876,27 @@
         <v>102</v>
       </c>
       <c r="AK99" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL99" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM99" t="s" s="2">
+        <v>596</v>
+      </c>
+      <c r="AN99" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO99" t="s" s="2">
         <v>597</v>
-      </c>
-      <c r="AL99" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM99" t="s" s="2">
-        <v>598</v>
-      </c>
-      <c r="AN99" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO99" t="s" s="2">
-        <v>599</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13928,13 +13922,13 @@
         <v>295</v>
       </c>
       <c r="L100" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="M100" t="s" s="2">
+        <v>600</v>
+      </c>
+      <c r="N100" t="s" s="2">
         <v>601</v>
-      </c>
-      <c r="M100" t="s" s="2">
-        <v>602</v>
-      </c>
-      <c r="N100" t="s" s="2">
-        <v>603</v>
       </c>
       <c r="O100" s="2"/>
       <c r="P100" t="s" s="2">
@@ -13984,7 +13978,7 @@
         <v>81</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>79</v>
@@ -14005,7 +13999,7 @@
         <v>81</v>
       </c>
       <c r="AM100" t="s" s="2">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="AN100" t="s" s="2">
         <v>81</v>
@@ -14016,10 +14010,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -14131,10 +14125,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -14248,10 +14242,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14367,10 +14361,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -14393,13 +14387,13 @@
         <v>81</v>
       </c>
       <c r="K104" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="L104" t="s" s="2">
+        <v>608</v>
+      </c>
+      <c r="M104" t="s" s="2">
         <v>609</v>
-      </c>
-      <c r="L104" t="s" s="2">
-        <v>610</v>
-      </c>
-      <c r="M104" t="s" s="2">
-        <v>611</v>
       </c>
       <c r="N104" s="2"/>
       <c r="O104" s="2"/>
@@ -14450,7 +14444,7 @@
         <v>81</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>90</v>
@@ -14468,24 +14462,24 @@
         <v>81</v>
       </c>
       <c r="AL104" t="s" s="2">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="AM104" t="s" s="2">
         <v>407</v>
       </c>
       <c r="AN104" t="s" s="2">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="AO104" t="s" s="2">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s" s="2">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -14511,13 +14505,13 @@
         <v>110</v>
       </c>
       <c r="L105" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="M105" t="s" s="2">
+        <v>615</v>
+      </c>
+      <c r="N105" t="s" s="2">
         <v>616</v>
-      </c>
-      <c r="M105" t="s" s="2">
-        <v>617</v>
-      </c>
-      <c r="N105" t="s" s="2">
-        <v>618</v>
       </c>
       <c r="O105" s="2"/>
       <c r="P105" t="s" s="2">
@@ -14546,10 +14540,10 @@
         <v>218</v>
       </c>
       <c r="Y105" t="s" s="2">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="Z105" t="s" s="2">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="AA105" t="s" s="2">
         <v>81</v>
@@ -14567,7 +14561,7 @@
         <v>81</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>79</v>
@@ -14588,7 +14582,7 @@
         <v>81</v>
       </c>
       <c r="AM105" t="s" s="2">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="AN105" t="s" s="2">
         <v>81</v>
@@ -14599,10 +14593,10 @@
     </row>
     <row r="106">
       <c r="A106" t="s" s="2">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -14628,13 +14622,13 @@
         <v>225</v>
       </c>
       <c r="L106" t="s" s="2">
+        <v>621</v>
+      </c>
+      <c r="M106" t="s" s="2">
+        <v>622</v>
+      </c>
+      <c r="N106" t="s" s="2">
         <v>623</v>
-      </c>
-      <c r="M106" t="s" s="2">
-        <v>624</v>
-      </c>
-      <c r="N106" t="s" s="2">
-        <v>625</v>
       </c>
       <c r="O106" s="2"/>
       <c r="P106" t="s" s="2">
@@ -14663,10 +14657,10 @@
         <v>336</v>
       </c>
       <c r="Y106" t="s" s="2">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="Z106" t="s" s="2">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="AA106" t="s" s="2">
         <v>81</v>
@@ -14684,7 +14678,7 @@
         <v>81</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>79</v>
@@ -14716,10 +14710,10 @@
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -14745,10 +14739,10 @@
         <v>256</v>
       </c>
       <c r="L107" t="s" s="2">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="M107" t="s" s="2">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="N107" s="2"/>
       <c r="O107" s="2"/>
@@ -14799,7 +14793,7 @@
         <v>81</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>79</v>
@@ -14831,10 +14825,10 @@
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14860,10 +14854,10 @@
         <v>544</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="M108" t="s" s="2">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="N108" s="2"/>
       <c r="O108" s="2"/>
@@ -14914,7 +14908,7 @@
         <v>81</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>79</v>
@@ -14929,27 +14923,27 @@
         <v>102</v>
       </c>
       <c r="AK108" t="s" s="2">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="AL108" t="s" s="2">
         <v>406</v>
       </c>
       <c r="AM108" t="s" s="2">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="AN108" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AO108" t="s" s="2">
-        <v>636</v>
+        <v>634</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14972,16 +14966,16 @@
         <v>81</v>
       </c>
       <c r="K109" t="s" s="2">
+        <v>636</v>
+      </c>
+      <c r="L109" t="s" s="2">
+        <v>637</v>
+      </c>
+      <c r="M109" t="s" s="2">
         <v>638</v>
       </c>
-      <c r="L109" t="s" s="2">
+      <c r="N109" t="s" s="2">
         <v>639</v>
-      </c>
-      <c r="M109" t="s" s="2">
-        <v>640</v>
-      </c>
-      <c r="N109" t="s" s="2">
-        <v>641</v>
       </c>
       <c r="O109" s="2"/>
       <c r="P109" t="s" s="2">
@@ -15031,7 +15025,7 @@
         <v>81</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>79</v>
@@ -15049,10 +15043,10 @@
         <v>81</v>
       </c>
       <c r="AL109" t="s" s="2">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="AM109" t="s" s="2">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="AN109" t="s" s="2">
         <v>81</v>

</xml_diff>